<commit_message>
[Codex] refactor: 分離地圖與 NPC 配置來源
</commit_message>
<xml_diff>
--- a/config/Excel/Zone_Stage_Drops.xlsx
+++ b/config/Excel/Zone_Stage_Drops.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="關卡掉落" sheetId="1" r:id="Rb4f920c8c3964d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="關卡掉落" sheetId="1" r:id="Re730e72ff4b14b72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -153,7 +153,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ZoneStageDropsTable" displayName="ZoneStageDropsTable" ref="A1:I17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ZoneStageDropsTable" displayName="ZoneStageDropsTable" ref="A1:I29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="地圖識別碼"/>
     <x:tableColumn id="2" name="最低關卡"/>
@@ -868,10 +868,358 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="18" t="str">
+        <x:v>god_battlefield</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="str">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="D18" s="18" t="str">
+        <x:v>53|48|47|10|3|1|0.08|0</x:v>
+      </x:c>
+      <x:c r="E18" s="18" t="str">
+        <x:v>11|1.7|0.6|0.1|0.08</x:v>
+      </x:c>
+      <x:c r="F18" s="18" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G18" s="18" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H18" s="18" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I18" s="18" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="18" t="str">
+        <x:v>god_battlefield</x:v>
+      </x:c>
+      <x:c r="B19" s="20" t="str">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="C19" s="20" t="str">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="D19" s="18" t="str">
+        <x:v>61|51|49|20|6|2|0.16|0</x:v>
+      </x:c>
+      <x:c r="E19" s="18" t="str">
+        <x:v>14|2.4|0.8|0.2|0.16</x:v>
+      </x:c>
+      <x:c r="F19" s="18" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G19" s="18" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H19" s="18" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I19" s="18" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="18" t="str">
+        <x:v>god_battlefield</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="str">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="str">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="D20" s="18" t="str">
+        <x:v>69|54|51|30|9|3|0.24|0</x:v>
+      </x:c>
+      <x:c r="E20" s="18" t="str">
+        <x:v>17|3.1|1|0.3|0.24</x:v>
+      </x:c>
+      <x:c r="F20" s="18" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G20" s="18" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H20" s="18" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I20" s="18" t="str">
+        <x:v>1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="18" t="str">
+        <x:v>god_battlefield</x:v>
+      </x:c>
+      <x:c r="B21" s="20" t="str">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C21" s="20" t="str">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="D21" s="18" t="str">
+        <x:v>77|57|53|40|12|4|0.32|0</x:v>
+      </x:c>
+      <x:c r="E21" s="18" t="str">
+        <x:v>20|3.8|1.2|0.4|0.32</x:v>
+      </x:c>
+      <x:c r="F21" s="18" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G21" s="18" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H21" s="18" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I21" s="18" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="18" t="str">
+        <x:v>god_chaos</x:v>
+      </x:c>
+      <x:c r="B22" s="20" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="20" t="str">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="D22" s="18" t="str">
+        <x:v>61|56|55|10|3|1|0.08|0</x:v>
+      </x:c>
+      <x:c r="E22" s="18" t="str">
+        <x:v>11|1.7|0.6|0.1|0.08</x:v>
+      </x:c>
+      <x:c r="F22" s="18" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G22" s="18" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H22" s="18" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I22" s="18" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="18" t="str">
+        <x:v>god_chaos</x:v>
+      </x:c>
+      <x:c r="B23" s="20" t="str">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="C23" s="20" t="str">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="D23" s="18" t="str">
+        <x:v>69|59|57|20|6|2|0.16|0</x:v>
+      </x:c>
+      <x:c r="E23" s="18" t="str">
+        <x:v>14|2.4|0.8|0.2|0.16</x:v>
+      </x:c>
+      <x:c r="F23" s="18" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G23" s="18" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H23" s="18" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I23" s="18" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="18" t="str">
+        <x:v>god_chaos</x:v>
+      </x:c>
+      <x:c r="B24" s="20" t="str">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="C24" s="20" t="str">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="D24" s="18" t="str">
+        <x:v>77|62|59|30|9|3|0.24|0</x:v>
+      </x:c>
+      <x:c r="E24" s="18" t="str">
+        <x:v>17|3.1|1|0.3|0.24</x:v>
+      </x:c>
+      <x:c r="F24" s="18" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G24" s="18" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H24" s="18" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I24" s="18" t="str">
+        <x:v>1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="18" t="str">
+        <x:v>god_chaos</x:v>
+      </x:c>
+      <x:c r="B25" s="20" t="str">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="C25" s="20" t="str">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="D25" s="18" t="str">
+        <x:v>85|65|61|40|12|4|0.32|0</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="str">
+        <x:v>20|3.8|1.2|0.4|0.32</x:v>
+      </x:c>
+      <x:c r="F25" s="18" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G25" s="18" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H25" s="18" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I25" s="18" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="18" t="str">
+        <x:v>god_sanctuary</x:v>
+      </x:c>
+      <x:c r="B26" s="20" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C26" s="20" t="str">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="D26" s="18" t="str">
+        <x:v>69|64|63|10|3|1|0.08|0</x:v>
+      </x:c>
+      <x:c r="E26" s="18" t="str">
+        <x:v>11|1.7|0.6|0.1|0.08</x:v>
+      </x:c>
+      <x:c r="F26" s="18" t="str">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G26" s="18" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H26" s="18" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I26" s="18" t="str">
+        <x:v>0.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="18" t="str">
+        <x:v>god_sanctuary</x:v>
+      </x:c>
+      <x:c r="B27" s="20" t="str">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="C27" s="20" t="str">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="D27" s="18" t="str">
+        <x:v>77|67|65|20|6|2|0.16|0</x:v>
+      </x:c>
+      <x:c r="E27" s="18" t="str">
+        <x:v>14|2.4|0.8|0.2|0.16</x:v>
+      </x:c>
+      <x:c r="F27" s="18" t="str">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G27" s="18" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H27" s="18" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I27" s="18" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="18" t="str">
+        <x:v>god_sanctuary</x:v>
+      </x:c>
+      <x:c r="B28" s="20" t="str">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="C28" s="20" t="str">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="D28" s="18" t="str">
+        <x:v>85|70|67|30|9|3|0.24|0</x:v>
+      </x:c>
+      <x:c r="E28" s="18" t="str">
+        <x:v>17|3.1|1|0.3|0.24</x:v>
+      </x:c>
+      <x:c r="F28" s="18" t="str">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="G28" s="18" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H28" s="18" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I28" s="18" t="str">
+        <x:v>1.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="18" t="str">
+        <x:v>god_sanctuary</x:v>
+      </x:c>
+      <x:c r="B29" s="20" t="str">
+        <x:v>601</x:v>
+      </x:c>
+      <x:c r="C29" s="20" t="str">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="D29" s="18" t="str">
+        <x:v>93|73|69|40|12|4|0.32|0</x:v>
+      </x:c>
+      <x:c r="E29" s="18" t="str">
+        <x:v>20|3.8|1.2|0.4|0.32</x:v>
+      </x:c>
+      <x:c r="F29" s="18" t="str">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G29" s="18" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H29" s="18" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I29" s="18" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc281add2368e431c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f636344bed54727"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>